<commit_message>
Refine AI (Price + Gender)
</commit_message>
<xml_diff>
--- a/Gift_Store_Data.xlsx
+++ b/Gift_Store_Data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\phamt\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\trung\Desktop\Trung_ERP\ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30845717-D3E7-4C9E-A0A0-8E01B8D4E19E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00FE97C2-9375-4B64-B93E-1CCF4AC98D9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9C4D112C-D429-4B6B-84FA-42C9A15777CD}"/>
+    <workbookView xWindow="6930" yWindow="1770" windowWidth="21600" windowHeight="11835" activeTab="1" xr2:uid="{9C4D112C-D429-4B6B-84FA-42C9A15777CD}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw Data" sheetId="1" r:id="rId1"/>
@@ -24,15 +24,6 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -862,7 +853,7 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -952,9 +943,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -992,7 +983,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1098,7 +1089,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1240,7 +1231,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>

</xml_diff>